<commit_message>
Corrige rodadas da semifinal da Libertadores
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/confrontos_fase_4_libertadores.xlsx
+++ b/libertadores/datasets_liberta/confrontos_fase_4_libertadores.xlsx
@@ -465,7 +465,7 @@
         <v>12</v>
       </c>
       <c r="D2">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s">
         <v>14</v>
@@ -491,7 +491,7 @@
         <v>13</v>
       </c>
       <c r="D3">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
         <v>15</v>
@@ -517,7 +517,7 @@
         <v>10</v>
       </c>
       <c r="D4">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
         <v>16</v>
@@ -543,7 +543,7 @@
         <v>11</v>
       </c>
       <c r="D5">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>

</xml_diff>